<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.003-05 Le toit rouge d'Amir
Réécriture vocale example4 : éclat de crochet, lunettes vécues.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.003-05.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.003-05.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cour de l'école</t>
+          <t>école, couloir, cour, crochets, craie, manteau rouge, crayons</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Amir, Nino, maman</t>
+          <t>Amir, Nino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut dessiner une maison au toit rouge pour maman. Le crayon rouge roule sous le banc. Nino le voit avec ses lunettes. Maman reçoit le dessin.</t>
+          <t>Un crochet penche vers le mur. Sur le métal, un éclat de crochet brille. Amir veut un toit rouge, maintenant. Nino arrive. Un rire commence. Nino se tait. Le crayon tape le sol. Amir refuse de foncer. Ils tiennent la feuille, à deux. Merci vécu. Le manteau glisse. L'éclat de crochet tient sur le métal.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le robinet de la cour laisse une goutte. Elle fait un rond sur le carreau. Les carreaux brillent encore. Ça sent le savon. Un bout de craie attend au sol. Maman pose une boîte sur le banc. Le bois du banc est froid. Dedans, des crayons. Tu as entendu la goutte, Amir ? Elle tombe. Oui. Tout doux. Amir pose le doigt sur le carreau. Le carreau est froid et lisse. En ce moment, Amir prend une feuille. Le papier est un peu rêche. Je dessine une maison. Avec un toit rouge. Pour toi, maman. J'aimerais beaucoup. Une porte, et un toit. Nino arrive près du banc. Nino a des lunettes. Nino a les cheveux courts. Il porte un manteau rouge. Nino, tu colories aussi. Tu colories avec moi ? Oui. Amir prend le crayon bleu. Nino prend le crayon jaune. Le bois des crayons est lisse. Le bleu fait un ciel. Le jaune fait un soleil. Le rouge, maintenant. Le crayon rouge roule. Il fait un petit bruit. Il glisse sous le banc. Il est parti. On peut le chercher. Tout doux, près des pieds.</t>
+          <t>Un crochet de manteau penche vers le mur. Le métal est froid, près de la porte. Ça cliquette, papa ! Tu l'entends, le petit bruit ? Oui, un clic. Dans le couloir, les crochets sentent le tissu. Sur le métal, un éclat de crochet brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Un bout de craie attend, côté cour. Il est court, un peu blanc. J'ai vu la craie. Elle est au sol, Amir ? Oui, papa. La feuille est rêche, sous la main. Elle gratte un peu. Papa pose une boîte près du banc. Dedans, des crayons, serrés. Les crayons sentent le papier, Amir ? Un peu, maman. En ce moment, Amir tient une feuille. Il veut un toit rouge, tout de suite. Je dessine une maison, maintenant ! Avec un toit rouge. Un toit rouge, pour maman ? Oui, papa. Tu veux le rouge, Amir ? Oui, le rouge. Nino arrive près des crochets. Ses pas font un bruit sec. Nino a des lunettes. Nino a les cheveux courts. Il porte un manteau rouge. Nino, tu poses le manteau ? Tu colories avec moi ? Oui. Nino accroche le manteau rouge. Le crochet penche un peu plus. Amir regarde les lunettes, trop longtemps. Un rire commence dans sa bouche. Nino ne dit rien. Le sourire de Nino disparaît. Tu prends le jaune, maintenant ! Nino recule d'un pas. Non. Oh. Amir prend le crayon rouge, tout seul. Le crayon roule hors de la feuille. Il tape le sol, trop vite. Ça fait un bruit dur. Un peu de craie colle au rouge. Il ne tient pas ! Il est tombé. L'éclat de crochet tremble, puis tient. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Amir ? Oui, papa. Tes mains sont froides, Amir ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le robinet de la cour laisse une goutte. Elle fait un rond sur le carreau. Les carreaux brillent encore. Ça sent le savon. Un bout de craie attend au sol. Maman pose une boîte sur le banc. Le bois du banc est froid. Dedans, des crayons. Tu as entendu la goutte, Amir ? Elle tombe. Oui. Tout doux. Amir pose le doigt sur le carreau. Le carreau est froid et lisse. En ce moment, Amir prend une feuille. Le papier est un peu rêche. Je dessine une maison. Avec un toit rouge. Pour toi, maman. J'aimerais beaucoup. Une porte, et un toit. Nino arrive près du banc. Nino a des lunettes. Nino a les cheveux courts. Il porte un manteau rouge. Nino, tu colories aussi. Tu colories avec moi ? Oui. Amir prend le crayon bleu. Nino prend le crayon jaune. Le bois des crayons est lisse. Le bleu fait un ciel. Le jaune fait un soleil. Le rouge, maintenant. Le crayon rouge roule. Il fait un petit bruit. Il glisse sous le banc. Il est parti. On peut le chercher. Tout doux, près des pieds.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un crochet de manteau penche vers le mur. Le métal est froid, près de la porte. Ça cliquette, papa ! Tu l'entends, le petit bruit ? Oui, un clic. Dans le couloir, les crochets sentent le tissu. Sur le métal, un &lt;emphasis level="moderate"&gt;éclat de crochet&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Un bout de craie attend, côté cour. Il est court, un peu blanc. J'ai vu la craie. Elle est au sol, Amir ? Oui, papa. La feuille est rêche, sous la main. Elle gratte un peu. Papa pose une boîte près du banc. Dedans, des crayons, serrés. Les crayons sentent le papier, Amir ? Un peu, maman. En ce moment, Amir tient une feuille. Il veut un toit rouge, tout de suite. Je dessine une maison, maintenant ! Avec un toit rouge. Un toit rouge, pour maman ? Oui, papa. Tu veux le rouge, Amir ? Oui, le rouge. Nino arrive près des crochets. Ses pas font un bruit sec. Nino a des lunettes. Nino a les cheveux courts. Il porte un manteau rouge. Nino, tu poses le manteau ? Tu colories avec moi ? Oui. Nino accroche le manteau rouge. Le crochet penche un peu plus. Amir regarde les lunettes, trop longtemps. Un rire commence dans sa bouche. Nino ne dit rien. Le sourire de Nino disparaît. Tu prends le jaune, maintenant ! Nino recule d'un pas. Non. Oh. Amir prend le crayon rouge, tout seul. Le crayon roule hors de la feuille. Il tape le sol, trop vite. Ça fait un bruit dur. Un peu de craie colle au rouge. Il ne tient pas ! Il est tombé. L'éclat de crochet tremble, puis tient. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Amir ? Oui, papa. Tes mains sont froides, Amir ? Un peu, maman.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Le matin, maman accompagne Alban à l'école. Dans la cour, un camarade arrive. Il a des lunettes. Il a les cheveux courts. Il porte un manteau rouge. Alban regarde. Un autre enfant laisse sortir un petit rire. Maman s'approche tout de suite. Maman dit : on ne va &lt;emphasis&gt;pas&lt;/emphasis&gt; rire de l'apparence. Les lunettes aident à voir. Les cheveux sont les cheveux. L'habit tient chaud. On joue. Alban hoche la tête. Il va vers le camarade. Alban dit : tu viens au bac à feuilles. Ils ramassent des feuilles. Plus tard, en classe, il y a des crayons. Un enfant regarde encore les lunettes. Alban dit : on ne va pas rire. On joue. Ils colorient. On ne rit pas des lunettes, des cheveux ou d'un habit. On ne va pas rire de l'apparence. On joue ensemble. [pause]</t>
+          <t>Un crochet de manteau penche vers le mur. Le métal est froid, près de la porte. Ça cliquette, papa ! Tu l'entends, le petit bruit ? Oui, un clic. Dans le couloir, les crochets sentent le tissu. Sur le métal, un &lt;emphasis&gt;éclat de crochet&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Un bout de craie attend, côté cour. Il est court, un peu blanc. J'ai vu la craie. Elle est au sol, Amir ? Oui, papa. La feuille est rêche, sous la main. Elle gratte un peu. Papa pose une boîte près du banc. Dedans, des crayons, serrés. Les crayons sentent le papier, Amir ? Un peu, maman. En ce moment, Amir tient une feuille. Il veut un toit rouge, tout de suite. Je dessine une maison, maintenant ! Avec un toit rouge. Un toit rouge, pour maman ? Oui, papa. Tu veux le rouge, Amir ? Oui, le rouge. Nino arrive près des crochets. Ses pas font un bruit sec. Nino a des lunettes. Nino a les cheveux courts. Il porte un manteau rouge. Nino, tu poses le manteau ? Tu colories avec moi ? Oui. Nino accroche le manteau rouge. Le crochet penche un peu plus. Amir regarde les lunettes, trop longtemps. Un rire commence dans sa bouche. Nino ne dit rien. Le sourire de Nino disparaît. Tu prends le jaune, maintenant ! Nino recule d'un pas. Non. Oh. Amir prend le crayon rouge, tout seul. Le crayon roule hors de la feuille. Il tape le sol, trop vite. Ça fait un bruit dur. Un peu de craie colle au rouge. Il ne tient pas ! Il est tombé. L'éclat de crochet tremble, puis tient. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Amir ? Oui, papa. Tes mains sont froides, Amir ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>éclat de crochet</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,49 +1321,76 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_un_toit_rouge_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le robinet de la cour laisse une goutte.
-narrateur|Elle fait un rond sur le carreau.
-narrateur|Les carreaux brillent encore.
-narrateur|Ça sent le savon.
-narrateur|Un bout de craie attend au sol.
-narrateur|Maman pose une boîte sur le banc.
-narrateur|Le bois du banc est froid.
-narrateur|Dedans, des crayons.
-maman|Tu as entendu la goutte, Amir ?
-enfant-m|Elle tombe.
-maman|Oui.
-maman|Tout doux.
-narrateur|Amir pose le doigt sur le carreau.
-narrateur|Le carreau est froid et lisse.
-narrateur|En ce moment, Amir prend une feuille.
-narrateur|Le papier est un peu rêche.
-enfant-m|Je dessine une maison.
+          <t>narrateur|Un crochet de manteau penche vers le mur.
+narrateur|Le métal est froid, près de la porte.
+enfant-m|Ça cliquette, papa !
+papa|Tu l'entends, le petit bruit ?
+enfant-m|Oui, un clic.
+narrateur|Dans le couloir, les crochets sentent le tissu.
+narrateur|Sur le métal, un éclat de crochet brille.
+enfant-m|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-m|Oui, un petit point.
+narrateur|Un bout de craie attend, côté cour.
+narrateur|Il est court, un peu blanc.
+enfant-m|J'ai vu la craie.
+papa|Elle est au sol, Amir ?
+enfant-m|Oui, papa.
+maman|La feuille est rêche, sous la main.
+enfant-m|Elle gratte un peu.
+narrateur|Papa pose une boîte près du banc.
+narrateur|Dedans, des crayons, serrés.
+maman|Les crayons sentent le papier, Amir ?
+enfant-m|Un peu, maman.
+narrateur|En ce moment, Amir tient une feuille.
+narrateur|Il veut un toit rouge, tout de suite.
+enfant-m|Je dessine une maison, maintenant !
 enfant-m|Avec un toit rouge.
-enfant-m|Pour toi, maman.
-maman|J'aimerais beaucoup.
-maman|Une porte, et un toit.
-narrateur|Nino arrive près du banc.
+papa|Un toit rouge, pour maman ?
+enfant-m|Oui, papa.
+maman|Tu veux le rouge, Amir ?
+enfant-m|Oui, le rouge.
+narrateur|Nino arrive près des crochets.
+narrateur|Ses pas font un bruit sec.
 narrateur|Nino a des lunettes.
 narrateur|Nino a les cheveux courts.
 narrateur|Il porte un manteau rouge.
-maman|Nino, tu colories aussi.
+papa|Nino, tu poses le manteau ?
 enfant-m|Tu colories avec moi ?
 copain|Oui.
-narrateur|Amir prend le crayon bleu.
-narrateur|Nino prend le crayon jaune.
-narrateur|Le bois des crayons est lisse.
-narrateur|Le bleu fait un ciel.
-narrateur|Le jaune fait un soleil.
-enfant-m|Le rouge, maintenant.
-narrateur|Le crayon rouge roule.
-narrateur|Il fait un petit bruit.
-narrateur|Il glisse sous le banc.
-enfant-m|Il est parti.
-maman|On peut le chercher.
-maman|Tout doux, près des pieds.</t>
+narrateur|Nino accroche le manteau rouge.
+narrateur|Le crochet penche un peu plus.
+narrateur|Amir regarde les lunettes, trop longtemps.
+narrateur|Un rire commence dans sa bouche.
+narrateur|Nino ne dit rien.
+narrateur|Le sourire de Nino disparaît.
+enfant-m|Tu prends le jaune, maintenant !
+narrateur|Nino recule d'un pas.
+copain|Non.
+enfant-m|Oh.
+narrateur|Amir prend le crayon rouge, tout seul.
+narrateur|Le crayon roule hors de la feuille.
+narrateur|Il tape le sol, trop vite.
+narrateur|Ça fait un bruit dur.
+narrateur|Un peu de craie colle au rouge.
+enfant-m|Il ne tient pas !
+copain|Il est tombé.
+narrateur|L'éclat de crochet tremble, puis tient.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Nino, Amir ?
+enfant-m|Oui, papa.
+maman|Tes mains sont froides, Amir ?
+enfant-m|Un peu, maman.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1400,22 +1427,22 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nino a des lunettes. Que fait-on ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nino a des &lt;emphasis level="moderate"&gt;lunettes&lt;/emphasis&gt;. Que fait-on ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le camarade a des lunettes. Que fait-on ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nino a des &lt;emphasis&gt;lunettes&lt;/emphasis&gt;. Que fait-on ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>jouer</t>
+          <t>pas rire</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>jouer | ensemble | chercher | crayon | on joue | pas rire</t>
+          <t>pas rire | on joue | jouer | pas rire apparence</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1430,7 +1457,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Nino voit le crayon. Que fait-on ?</t>
+          <t>Pas rire. Nino a des lunettes. Que fait-on ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1468,7 +1495,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1479,7 +1506,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1494,34 +1521,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>lunettes</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1536,17 +1567,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=pas_rire_nino_a_des_lunettes; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1579,17 +1610,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nino se penche près du banc. Il voit un bout de rouge. Là. Tout au fond. Amir allonge le bras. La poussière du sol est fine. Il rattrape le crayon rouge. Le bois est un peu froid. Merci, Amir. Merci, Nino. J'ai le toit. Nino a vu le crayon. Le toit peut se faire. Amir dessine le toit. Le rouge est vif sur le papier. Il est beau. C'est pour maman.</t>
+          <t>Amir veut le toit rouge, tout de suite. Je colorie, maintenant ! Il avance trop vite vers Nino. Les mots se bousculent dans sa bouche. Non. Nino reste un peu plus loin. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le crayon, un instant. Il écoute le clic du crochet. Tu veux le toit avec Nino ? Papa reste à la même hauteur. Tu tiens la feuille ? Nino ne dit rien, d'abord. Il pose les mains sur le papier. Je la tiens. D'accord. Merci, Amir. Papa a vu les deux, près du banc. La craie colle un peu, sous les doigts. Elle est sèche. Ils essuient le crayon sur le banc. Nino tient la feuille, plus près. Le crayon redevient plus ferme, cette fois. Il tient ! Oui. Tu le vois, le rouge ? Oui, papa. Le ciel, Nino ? J'y vais. Amir trace, sans se presser. Nino suit le trait des yeux. Nino pose le jaune, une fois. Le soleil. Le ciel. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On reste près du banc ? Oui. Tes mains sont au chaud ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nino se penche près du banc. Il voit un bout de rouge. Là. Tout au fond. Amir allonge le bras. La poussière du sol est fine. Il rattrape le crayon rouge. Le bois est un peu froid. Merci, Amir. Merci, Nino. J'ai le toit. Nino a vu le crayon. Le toit peut se faire. Amir dessine le toit. Le rouge est vif sur le papier. Il est beau. C'est pour maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir veut le toit rouge, tout de suite. Je colorie, maintenant ! Il avance trop vite vers Nino. Les mots se bousculent dans sa bouche. Non. Nino reste un peu plus loin. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le crayon, un instant. Il écoute le clic du crochet. Tu veux le toit avec Nino ? Papa reste à la même hauteur. Tu tiens la &lt;emphasis level="moderate"&gt;feuille&lt;/emphasis&gt; ? Nino ne dit rien, d'abord. Il pose les mains sur le papier. Je la tiens. D'accord. Merci, Amir. Papa a vu les deux, près du banc. La craie colle un peu, sous les doigts. Elle est sèche. Ils essuient le crayon sur le banc. Nino tient la feuille, plus près. Le crayon redevient plus ferme, cette fois. Il tient ! Oui. Tu le vois, le rouge ? Oui, papa. Le ciel, Nino ? J'y vais. Amir trace, sans se presser. Nino suit le trait des yeux. Nino pose le jaune, une fois. Le soleil. Le ciel. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On reste près du banc ? Oui. Tes mains sont au chaud ? Un peu, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Alban a entendu maman. On ne va &lt;emphasis&gt;pas&lt;/emphasis&gt; rire de l'apparence. Alban a invité le camarade. Ils ont joué. [pause]</t>
+          <t>Amir veut le toit rouge, tout de suite. Je colorie, maintenant ! Il avance trop vite vers Nino. Les mots se bousculent dans sa bouche. Non. Nino reste un peu plus loin. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le crayon, un instant. Il écoute le clic du crochet. Tu veux le toit avec Nino ? Papa reste à la même hauteur. Tu tiens la &lt;emphasis&gt;feuille&lt;/emphasis&gt; ? Nino ne dit rien, d'abord. Il pose les mains sur le papier. Je la tiens. D'accord. Merci, Amir. Papa a vu les deux, près du banc. La craie colle un peu, sous les doigts. Elle est sèche. Ils essuient le crayon sur le banc. Nino tient la feuille, plus près. Le crayon redevient plus ferme, cette fois. Il tient ! Oui. Tu le vois, le rouge ? Oui, papa. Le ciel, Nino ? J'y vais. Amir trace, sans se presser. Nino suit le trait des yeux. Nino pose le jaune, une fois. Le soleil. Le ciel. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On reste près du banc ? Oui. Tes mains sont au chaud ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1636,7 +1667,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1644,10 +1675,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1670,30 +1701,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>feuille</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1702,10 +1733,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1718,28 +1749,60 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=ils_tiennent_la_feuille_a_deux; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nino se penche près du banc.
-narrateur|Il voit un bout de rouge.
-copain|Là.
-copain|Tout au fond.
-narrateur|Amir allonge le bras.
-narrateur|La poussière du sol est fine.
-narrateur|Il rattrape le crayon rouge.
-narrateur|Le bois est un peu froid.
-maman|Merci, Amir.
-maman|Merci, Nino.
-enfant-m|J'ai le toit.
-maman|Nino a vu le crayon.
-maman|Le toit peut se faire.
-narrateur|Amir dessine le toit.
-narrateur|Le rouge est vif sur le papier.
-copain|Il est beau.
-enfant-m|C'est pour maman.</t>
+          <t>narrateur|Amir veut le toit rouge, tout de suite.
+enfant-m|Je colorie, maintenant !
+narrateur|Il avance trop vite vers Nino.
+narrateur|Les mots se bousculent dans sa bouche.
+copain|Non.
+narrateur|Nino reste un peu plus loin.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Amir refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe le crayon, un instant.
+narrateur|Il écoute le clic du crochet.
+papa|Tu veux le toit avec Nino ?
+narrateur|Papa reste à la même hauteur.
+enfant-m|Tu tiens la feuille ?
+narrateur|Nino ne dit rien, d'abord.
+narrateur|Il pose les mains sur le papier.
+copain|Je la tiens.
+enfant-m|D'accord.
+papa|Merci, Amir.
+narrateur|Papa a vu les deux, près du banc.
+maman|La craie colle un peu, sous les doigts.
+enfant-m|Elle est sèche.
+narrateur|Ils essuient le crayon sur le banc.
+narrateur|Nino tient la feuille, plus près.
+narrateur|Le crayon redevient plus ferme, cette fois.
+enfant-m|Il tient !
+copain|Oui.
+papa|Tu le vois, le rouge ?
+enfant-m|Oui, papa.
+maman|Le ciel, Nino ?
+copain|J'y vais.
+narrateur|Amir trace, sans se presser.
+narrateur|Nino suit le trait des yeux.
+narrateur|Nino pose le jaune, une fois.
+copain|Le soleil.
+enfant-m|Le ciel.
+narrateur|Le ventre d'Amir se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près du banc ?
+enfant-m|Oui.
+maman|Tes mains sont au chaud ?
+enfant-m|Un peu, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>crayons</t>
         </is>
       </c>
     </row>
@@ -1766,17 +1829,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>La maison a un toit rouge. Le soleil est jaune. Le ciel est bleu. Une porte. Et une fenêtre. Bravo. Vous avez colorié ensemble. Amir tend la feuille. C'est pour toi. Je la prends. Le toit est bien rouge. Maman souffle un peu dessus. Le crayon sèche. Le papier sent encore le bois. La goutte tombe encore. Oui. On l'entend. Nino range le crayon jaune. Amir range le crayon rouge. La boîte se ferme. Ça fait clic. Le dessin est à moi, maintenant. Oui. Pour la cuisine.</t>
+          <t>Amir trace le toit, plus vite. La porte. La fenêtre. Le manteau rouge bouge. Le crochet penche. Les lunettes restent sur le nez. Le rouge, maintenant ! Il colorie trop vite, tout de suite. Il regarde les lunettes, trop longtemps. Un rire revient dans sa bouche. Attends. Nino lâche la feuille. Le manteau glisse du crochet. Ça tombe ! Amir avance les mains, trop vite. Le pied part vers le papier. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le manteau, un instant. Il écoute le clic du crochet. Sur le métal, un éclat de crochet luit. Là, sur le crochet. Tu tiens la feuille, Nino ? Nino ne dit rien. Il reprend le papier, sans parler. Oui. Ils accrochent le manteau, sans se presser. Amir colorie, tout près de Nino. Nino pose le jaune. Le soleil ! Le toit ! Tu as fini le rouge ? Oui, papa. Le manteau est chaud, Nino ? Un peu. Le crayon se pose dans la boîte. On reverse les rôles ? À toi le jaune. Nino prend le rouge à son tour. Amir pose le bleu. Ses doigts font un trait. C'est plus facile. Le trait est net ? Oui, papa. Un rayon passe près des crochets. Il allume le manteau.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>La maison a un toit rouge. Le soleil est jaune. Le ciel est bleu. Une porte. Et une fenêtre. Bravo. Vous avez colorié ensemble. Amir tend la feuille. C'est pour toi. Je la prends. Le toit est bien rouge. Maman souffle un peu dessus. Le crayon sèche. Le papier sent encore le bois. La goutte tombe encore. Oui. On l'entend. Nino range le crayon jaune. Amir range le crayon rouge. La boîte se ferme. Ça fait clic. Le dessin est à moi, maintenant. Oui. Pour la cuisine.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir trace le toit, plus vite. La porte. La fenêtre. Le manteau rouge bouge. Le crochet penche. Les lunettes restent sur le nez. Le rouge, maintenant ! Il colorie trop vite, tout de suite. Il regarde les lunettes, trop longtemps. Un rire revient dans sa bouche. Attends. Nino lâche la feuille. Le manteau glisse du crochet. Ça tombe ! Amir avance les mains, trop vite. Le pied part vers le papier. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le manteau, un instant. Il écoute le clic du crochet. Sur le métal, un &lt;emphasis level="moderate"&gt;éclat de crochet&lt;/emphasis&gt; luit. Là, sur le crochet. Tu tiens la feuille, Nino ? Nino ne dit rien. Il reprend le papier, sans parler. Oui. Ils accrochent le manteau, sans se presser. Amir colorie, tout près de Nino. Nino pose le jaune. Le soleil ! Le toit ! Tu as fini le rouge ? Oui, papa. Le manteau est chaud, Nino ? Un peu. Le crayon se pose dans la boîte. On reverse les rôles ? À toi le jaune. Nino prend le rouge à son tour. Amir pose le bleu. Ses doigts font un trait. C'est plus facile. Le trait est net ? Oui, papa. Un rayon passe près des crochets. Il allume le manteau.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman revient près du portail. Alban et le camarade se disent à de&lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Amir trace le toit, plus vite. La porte. La fenêtre. Le manteau rouge bouge. Le crochet penche. Les lunettes restent sur le nez. Le rouge, maintenant ! Il colorie trop vite, tout de suite. Il regarde les lunettes, trop longtemps. Un rire revient dans sa bouche. Attends. Nino lâche la feuille. Le manteau glisse du crochet. Ça tombe ! Amir avance les mains, trop vite. Le pied part vers le papier. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le manteau, un instant. Il écoute le clic du crochet. Sur le métal, un &lt;emphasis&gt;éclat de crochet&lt;/emphasis&gt; luit. Là, sur le crochet. Tu tiens la feuille, Nino ? Nino ne dit rien. Il reprend le papier, sans parler. Oui. Ils accrochent le manteau, sans se presser. Amir colorie, tout près de Nino. Nino pose le jaune. Le soleil ! Le toit ! Tu as fini le rouge ? Oui, papa. Le manteau est chaud, Nino ? Un peu. Le crayon se pose dans la boîte. On reverse les rôles ? À toi le jaune. Nino prend le rouge à son tour. Amir pose le bleu. Ses doigts font un trait. C'est plus facile. Le trait est net ? Oui, papa. Un rayon passe près des crochets. Il allume le manteau. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1823,7 +1886,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1831,10 +1894,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1857,30 +1920,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de crochet</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1889,10 +1952,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1903,33 +1966,66 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_retrouve_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|La maison a un toit rouge.
-narrateur|Le soleil est jaune.
-narrateur|Le ciel est bleu.
-enfant-m|Une porte.
-copain|Et une fenêtre.
-maman|Bravo.
-maman|Vous avez colorié ensemble.
-narrateur|Amir tend la feuille.
-enfant-m|C'est pour toi.
-maman|Je la prends.
-maman|Le toit est bien rouge.
-narrateur|Maman souffle un peu dessus.
-narrateur|Le crayon sèche.
-narrateur|Le papier sent encore le bois.
-enfant-m|La goutte tombe encore.
-maman|Oui.
-maman|On l'entend.
-narrateur|Nino range le crayon jaune.
-narrateur|Amir range le crayon rouge.
-narrateur|La boîte se ferme.
-narrateur|Ça fait clic.
-maman|Le dessin est à moi, maintenant.
-enfant-m|Oui.
-enfant-m|Pour la cuisine.</t>
+          <t>narrateur|Amir trace le toit, plus vite.
+copain|La porte.
+enfant-m|La fenêtre.
+narrateur|Le manteau rouge bouge.
+narrateur|Le crochet penche.
+narrateur|Les lunettes restent sur le nez.
+enfant-m|Le rouge, maintenant !
+narrateur|Il colorie trop vite, tout de suite.
+narrateur|Il regarde les lunettes, trop longtemps.
+narrateur|Un rire revient dans sa bouche.
+copain|Attends.
+narrateur|Nino lâche la feuille.
+narrateur|Le manteau glisse du crochet.
+enfant-m|Ça tombe !
+narrateur|Amir avance les mains, trop vite.
+narrateur|Le pied part vers le papier.
+narrateur|Puis il s'arrête net.
+narrateur|Amir refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe le manteau, un instant.
+narrateur|Il écoute le clic du crochet.
+narrateur|Sur le métal, un éclat de crochet luit.
+enfant-m|Là, sur le crochet.
+enfant-m|Tu tiens la feuille, Nino ?
+narrateur|Nino ne dit rien.
+narrateur|Il reprend le papier, sans parler.
+copain|Oui.
+narrateur|Ils accrochent le manteau, sans se presser.
+narrateur|Amir colorie, tout près de Nino.
+narrateur|Nino pose le jaune.
+copain|Le soleil !
+enfant-m|Le toit !
+papa|Tu as fini le rouge ?
+enfant-m|Oui, papa.
+maman|Le manteau est chaud, Nino ?
+copain|Un peu.
+narrateur|Le crayon se pose dans la boîte.
+papa|On reverse les rôles ?
+copain|À toi le jaune.
+narrateur|Nino prend le rouge à son tour.
+narrateur|Amir pose le bleu.
+narrateur|Ses doigts font un trait.
+enfant-m|C'est plus facile.
+papa|Le trait est net ?
+enfant-m|Oui, papa.
+maman|Un rayon passe près des crochets.
+enfant-m|Il allume le manteau.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>crayons</t>
         </is>
       </c>
     </row>
@@ -1956,17 +2052,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le dessin est dans les mains de maman. Le toit rouge brille un peu. On l'a fini. Oui. Vous avez colorié la maison. Le robinet laisse encore une goutte.</t>
+          <t>Ils restent près des crochets. Maman essuie un peu de craie. On a eu le toit rouge, papa. Tu l'as vu, toi ? Oui, sur la feuille. On est bien, ici. Amir tapote le papier du doigt. Il a une trace de craie. Tu la vois, la trace ? Oui, maman. La feuille est restée, Amir. Oui, avec Nino. La feuille est restée. Ça sent le crayon, un peu tiède. Et le manteau, maman. Oui, dans l'air. Le manteau rouge reste au crochet. Un éclat de crochet tient sur le métal.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le dessin est dans les mains de maman. Le toit rouge brille un peu. On l'a fini. Oui. Vous avez colorié la maison. Le robinet laisse encore une goutte.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près des crochets. Maman essuie un peu de craie. On a eu le toit rouge, papa. Tu l'as vu, toi ? Oui, sur la feuille. On est bien, ici. Amir tapote le papier du doigt. Il a une trace de craie. Tu la vois, la trace ? Oui, maman. La feuille est restée, Amir. Oui, avec Nino. La feuille est restée. Ça sent le crayon, un peu tiède. Et le manteau, maman. Oui, dans l'air. Le manteau rouge reste au crochet. Un &lt;emphasis level="moderate"&gt;éclat de crochet&lt;/emphasis&gt; tient sur le métal.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près des crochets. Maman essuie un peu de craie. On a eu le toit rouge, papa. Tu l'as vu, toi ? Oui, sur la feuille. On est bien, ici. Amir tapote le papier du doigt. Il a une trace de craie. Tu la vois, la trace ? Oui, maman. La feuille est restée, Amir. Oui, avec Nino. La feuille est restée. Ça sent le crayon, un peu tiède. Et le manteau, maman. Oui, dans l'air. Le manteau rouge reste au crochet. Un &lt;emphasis&gt;éclat de crochet&lt;/emphasis&gt; tient sur le métal.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2013,18 +2109,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2033,12 +2129,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2047,17 +2143,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de crochet</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2066,11 +2166,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2079,29 +2179,50 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_metal; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le dessin est dans les mains de maman.
-narrateur|Le toit rouge brille un peu.
-enfant-m|On l'a fini.
-maman|Oui.
-maman|Vous avez colorié la maison.
-narrateur|Le robinet laisse encore une goutte.</t>
+          <t>narrateur|Ils restent près des crochets.
+narrateur|Maman essuie un peu de craie.
+enfant-m|On a eu le toit rouge, papa.
+papa|Tu l'as vu, toi ?
+enfant-m|Oui, sur la feuille.
+maman|On est bien, ici.
+narrateur|Amir tapote le papier du doigt.
+enfant-m|Il a une trace de craie.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|La feuille est restée, Amir.
+enfant-m|Oui, avec Nino.
+copain|La feuille est restée.
+narrateur|Ça sent le crayon, un peu tiède.
+enfant-m|Et le manteau, maman.
+maman|Oui, dans l'air.
+narrateur|Le manteau rouge reste au crochet.
+narrateur|Un éclat de crochet tient sur le métal.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>crochets</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2207,6 +2328,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>